<commit_message>
Importeren van correlatie invoer nu compleet
</commit_message>
<xml_diff>
--- a/geoprob_pipe/questionnaire/parameter_input/parameter_input_template.xlsx
+++ b/geoprob_pipe/questionnaire/parameter_input/parameter_input_template.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\geoprob_pipe\pre_processing\parameter_input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CP\git_clones\GeoProb-Pipe\GeoProb-PipeV2\GeoProb-Pipe\geoprob_pipe\questionnaire\parameter_input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD450CE-CDCB-41F7-AEF9-46B581B15214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D444FC-1AE4-40FF-A4C0-E3A13FFEE251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="725" activeTab="4" xr2:uid="{4072986C-855A-4E04-BDA4-92C994E74780}"/>
   </bookViews>
   <sheets>
     <sheet name="Geohydrologisch model" sheetId="1" r:id="rId1"/>
     <sheet name="Scenario invoer" sheetId="3" r:id="rId2"/>
     <sheet name="Parameter invoer" sheetId="2" r:id="rId3"/>
     <sheet name="Fragility values" sheetId="5" r:id="rId4"/>
-    <sheet name="Bronnen" sheetId="4" r:id="rId5"/>
+    <sheet name="Correlatie invoer" sheetId="7" r:id="rId5"/>
+    <sheet name="Bronnen" sheetId="4" r:id="rId6"/>
+    <sheet name="Additonele uitleg" sheetId="6" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Geohydrologisch model'!$A$6:$E$6</definedName>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="90">
   <si>
     <t>parameter</t>
   </si>
@@ -261,6 +263,62 @@
   </si>
   <si>
     <t>distribution_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optioneel invullen voor log_normal en normal.
+Momenteel nog niet geïmplementeerd. </t>
+  </si>
+  <si>
+    <t>Maximum</t>
+  </si>
+  <si>
+    <t>Minimum</t>
+  </si>
+  <si>
+    <t>(1)</t>
+  </si>
+  <si>
+    <t>Fragility values ref</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De fragility values worden voornamelijk gebruikt om handmatige overschrijdingsfrequentielijnen te gebruiken. Dit is bijvoorbeeld handig voor ontwerpprojecten. </t>
+  </si>
+  <si>
+    <t>(2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indien je een csv-bestand opgeeft, gebruik dan als referentie de naam van het csv-bestand. GeoProb-Pipe zoekt het csv-bestand vervolgens in de map 'frag_csv_files'. Indien GeoProb-Pipe het bestand niet kan terug vinden zal hij je exact aangeven waar je het bestand moet neerzetten. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Het wordt aangeraden om handmatige fragility values op te geven in het tabblad 'Fragility values' in plaats van in aparte csv-bestanden. Dit is omdat de csv-bestand niet opgeslagen worden in het GeoProb-Pipe-bestand. </t>
+  </si>
+  <si>
+    <t>(3)</t>
+  </si>
+  <si>
+    <t>Referentie naar de fragility values. Dat is, de naam van de Hydra-NL-locatie of een handmatige invoer in tabblad 'Fragility values' of een csv-bestand. 
+Zie additionele uitleg in nummers (1-3).</t>
+  </si>
+  <si>
+    <t>Parameter A</t>
+  </si>
+  <si>
+    <t>Parameter B</t>
+  </si>
+  <si>
+    <t>Correlatie</t>
+  </si>
+  <si>
+    <t>parameter_a</t>
+  </si>
+  <si>
+    <t>parameter_b</t>
+  </si>
+  <si>
+    <t>correlation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correlatie op trajectniveau. Getal tussen 0 en 1, waarbij 1 volledig gecorreleerd. GeoProb-Pipe hanteert standaard, 0 wanneer je geen correlatie opgeeft. </t>
   </si>
 </sst>
 </file>
@@ -318,7 +376,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -355,6 +413,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -369,7 +433,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -441,6 +505,27 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -990,9 +1075,8 @@
     <col min="6" max="6" width="21.5546875" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.88671875" style="11" customWidth="1"/>
     <col min="8" max="8" width="12.33203125" style="11" customWidth="1"/>
-    <col min="9" max="9" width="8.44140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.88671875" style="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.6640625" style="11" customWidth="1"/>
+    <col min="9" max="10" width="15.44140625" style="11" customWidth="1"/>
+    <col min="11" max="11" width="21.44140625" style="11" customWidth="1"/>
     <col min="12" max="12" width="38.88671875" style="11" customWidth="1"/>
     <col min="13" max="13" width="66" style="11" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="11"/>
@@ -1021,9 +1105,15 @@
       <c r="H1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="I1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>76</v>
+      </c>
       <c r="L1" s="8" t="s">
         <v>29</v>
       </c>
@@ -1056,9 +1146,15 @@
       <c r="H2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="16"/>
-      <c r="J2" s="16"/>
-      <c r="K2" s="16"/>
+      <c r="I2" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>82</v>
+      </c>
       <c r="L2" s="16" t="s">
         <v>33</v>
       </c>
@@ -1201,6 +1297,62 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C10C9D3-628F-4899-B2B7-5991A202D351}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="35.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="28" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="55.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="29"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="30" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEE6525A-680B-4461-9F3B-3E1CE43163B1}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1333,4 +1485,43 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{330664B7-9142-40FB-8A8A-37B16B47325A}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3.109375" style="27" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="138.33203125" style="27" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.88671875" style="27"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>